<commit_message>
feat!: new input parameter in file conductor_grid.xlsx
Number of evenly spaced elements used in adaptive mesh to split each element
that need refinement. So, if an element of lenght 1 m should be refined and
NELEMS_REFINEMEN = 2, the element will be splitted into two elements of lenght
0.5 m each. This parameters is used only if flag ITYMSH is set to 2 or 3.

BREAKING CHANGES

    Input files without this parameter will raise an error.
    With this input parameter the adaptive mesh is officially introduced in OpenSc2.
    Flag ITYMSH can now assume values 2 and 3 and work correctly adapting the mesh at
    each thermal hydraulic time step.

modified:   input_files/input_file_template/template_conductor_grid.xlsx
</commit_message>
<xml_diff>
--- a/source_code/input_files/input_file_template/template_conductor_grid.xlsx
+++ b/source_code/input_files/input_file_template/template_conductor_grid.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\daniele.placido\3D Objects\OPENSC2\source_code\input_files\input_file_template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniele.Placido\3D Objects\OPENSC2\source_code\input_files\input_file_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD0AD516-560B-42B3-8BF9-DA6910C10E76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA91605-2119-4BBC-8F1D-8C39A707C068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GRID" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="25">
   <si>
     <t>NELEMS</t>
   </si>
@@ -106,6 +106,12 @@
   </si>
   <si>
     <t>size increase ratio for the spatial mesh, used for the region to the right of the refined region.</t>
+  </si>
+  <si>
+    <t>NELEMS_REFINEMENT</t>
+  </si>
+  <si>
+    <t>Number of evenly spaced elements used in adaptive mesh to split each element that need refinement. So, if an element of lenght 1 m should be refined and NELEMS_REFINEMEN = 2, the element will be splitted into two elements of lenght 0.5 m each. This parameters is used only if flag ITYMSH is set to 2 or 3.</t>
   </si>
 </sst>
 </file>
@@ -215,7 +221,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="CONDUCTOR_files"/>
@@ -243,7 +249,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="TRANSIENT"/>
@@ -271,9 +277,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -311,7 +317,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -417,7 +423,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -559,7 +565,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -567,18 +573,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" style="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="60.42578125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.54296875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.1796875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="60.453125" style="9" customWidth="1"/>
     <col min="5" max="5" width="14" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.85546875" style="2"/>
+    <col min="6" max="16384" width="8.81640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="str">
         <f>[1]CONDUCTOR_files!$A$1</f>
         <v>CONDUCTOR</v>
@@ -594,7 +600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="6"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -603,7 +609,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="str">
         <f>[2]TRANSIENT!A$2</f>
         <v>Variable name</v>
@@ -625,7 +631,7 @@
         <v>CONDUCTOR_1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -639,7 +645,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
@@ -656,7 +662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
@@ -673,7 +679,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>7</v>
       </c>
@@ -691,7 +697,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>8</v>
       </c>
@@ -708,7 +714,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>9</v>
       </c>
@@ -725,7 +731,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
         <v>10</v>
       </c>
@@ -742,7 +748,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>19</v>
       </c>
@@ -759,7 +765,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
         <v>21</v>
       </c>
@@ -776,9 +782,9 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>2</v>
@@ -787,9 +793,26 @@
         <v>3</v>
       </c>
       <c r="D13" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E14" s="3">
         <v>10001</v>
       </c>
     </row>

</xml_diff>

<commit_message>
doc: update documentation in conductor_grid.xlsx
Updated documentation in input file conductor_grid.xlsx as follows.
    * Flag ITYMSH can assume 2 new values
        2: adaptive grid from initial uniform grid
        3: adaptive grid from initial refined grid
    * Added detailed docstring for input parameter NELEMS
    * Described the behavior of the code according to the value of flag ITYMSH
        for the following input parameters: NELREF, XBREFI, XEREFI, SIZMIN,
        SIZMAX, DXINCRE_LEFT, DXINCRE_RIGHT.

modified:   input_files/input_file_template/template_conductor_grid.xlsx
</commit_message>
<xml_diff>
--- a/source_code/input_files/input_file_template/template_conductor_grid.xlsx
+++ b/source_code/input_files/input_file_template/template_conductor_grid.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniele.Placido\3D Objects\OPENSC2\source_code\input_files\input_file_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA91605-2119-4BBC-8F1D-8C39A707C068}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F688EA-3854-450B-A0C9-7C3483614CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GRID" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
   <si>
     <t>NELEMS</t>
   </si>
@@ -72,46 +72,49 @@
     <t>SIZMAX</t>
   </si>
   <si>
-    <t xml:space="preserve"> number of spatial elements in the refined zone                                                                                                 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">starting point of the refined zone                                                                          </t>
-  </si>
-  <si>
-    <t xml:space="preserve">end point of the refined zone                                                                          </t>
-  </si>
-  <si>
-    <t xml:space="preserve">minimum spatial mesh size (if refined)                                                                                                                                      </t>
-  </si>
-  <si>
-    <t xml:space="preserve">maximum spatial mesh size (if refined)                                                                                                                                      </t>
-  </si>
-  <si>
-    <t xml:space="preserve">flag for mesh type: 0 = fixed and uniform; 1 = fixed refined; 3 = adapted with initial refinement; - 1 from file; in this case the z coordinates of the conductor components must be exactly the same for each conudctor component objets.                                                                     </t>
-  </si>
-  <si>
     <t>MAXNOD</t>
   </si>
   <si>
-    <t xml:space="preserve"> maximum number of nodes for conductor spatial discretization</t>
-  </si>
-  <si>
     <t>DXINCRE_LEFT</t>
   </si>
   <si>
-    <t>size increase ratio for the spatial mesh, used for the region to the left of the refined region.</t>
-  </si>
-  <si>
     <t>DXINCRE_RIGHT</t>
   </si>
   <si>
-    <t>size increase ratio for the spatial mesh, used for the region to the right of the refined region.</t>
-  </si>
-  <si>
     <t>NELEMS_REFINEMENT</t>
   </si>
   <si>
     <t>Number of evenly spaced elements used in adaptive mesh to split each element that need refinement. So, if an element of lenght 1 m should be refined and NELEMS_REFINEMEN = 2, the element will be splitted into two elements of lenght 0.5 m each. This parameters is used only if flag ITYMSH is set to 2 or 3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum spatial mesh size. This input argument is relevant if flag ITYMSH is set to 1 (static refined grid), 2 (adaptive grid from initial uniform grid) or 3 (adaptive grid from initial refined grid).                                                                                                                                  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flag to select the grid type: 0 = static and uniform grid; 1 = static and refined grid; 2 = adaptive grid from intial uniform grid; 3 = adaptive grid from initial refined grid; - 1 grid loaded from file; in this case the z coordinates of the conductor components must be exactly the same for each conudctor component objets.                                                                     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum spatial mesh size. This input argument is relevant if flag ITYMSH is set to 1 (static refined grid), 2 (adaptive grid from initial uniform grid) or 3 (adaptive grid from initial refined grid).                                                                                                                                 </t>
+  </si>
+  <si>
+    <t>Number of spatial elements in the refined zone; used if flag ITYMSH is set to  1 (static refined grid) or 3 (adaptive grid from initial refined grid).</t>
+  </si>
+  <si>
+    <t>Starting point of the refined zone; used if flag ITYMSH is set to  1 (static refined grid) or 3 (adaptive grid from initial refined grid).</t>
+  </si>
+  <si>
+    <t>End point of the refined zone; used if flag ITYMSH is set to  1 (static refined grid) or 3 (adaptive grid from initial refined grid).</t>
+  </si>
+  <si>
+    <t>Size increase ratio for the spatial mesh, used for the region to the left of the refined region. This input argument is used if flag ITYMSH is set to  1 (static refined grid) or 3 (adaptive grid from initial refined grid).</t>
+  </si>
+  <si>
+    <t>Size increase ratio for the spatial mesh, used for the region to the right of the refined region. This input argument is used if flag ITYMSH is set to  1 (static refined grid) or 3 (adaptive grid from initial refined grid).</t>
+  </si>
+  <si>
+    <t>Maximum number of nodes for conductor spatial discretization</t>
+  </si>
+  <si>
+    <t>Number of elements used to discretize the mesh. If grid is static (ITYMSH = 0 or ITYMNSH = 1), NELEMS is the number of nodes used in the whole simulation. If grid is adaptive (ITYMSH = 2 or ITYMNSH = 3), NELEMS is used to evaluate the initial mesh and to identify the hard nodes, i.e. the set of minimum nodes on which the solution will be available. The number of nodes can be increased by the algorithm up to MAXNOD locally adding soft nodes in regions with strong gradients (nearby the quench fronts). If grid is loaded from auxiliary input files (ITYMNSH = -1), this parameter is ignored.</t>
   </si>
 </sst>
 </file>
@@ -631,9 +634,9 @@
         <v>CONDUCTOR_1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -641,13 +644,16 @@
       <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
+      <c r="D4" s="9" t="s">
+        <v>17</v>
+      </c>
       <c r="E4" s="11">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="58" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>2</v>
@@ -656,13 +662,13 @@
         <v>3</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E5" s="11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
@@ -673,13 +679,13 @@
         <v>3</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E6" s="11">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>7</v>
       </c>
@@ -690,14 +696,14 @@
         <v>4</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E7" s="10">
         <f>26</f>
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>8</v>
       </c>
@@ -708,13 +714,13 @@
         <v>4</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E8" s="10">
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>9</v>
       </c>
@@ -725,13 +731,13 @@
         <v>4</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E9" s="10">
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
         <v>10</v>
       </c>
@@ -742,15 +748,15 @@
         <v>4</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E10" s="10">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>2</v>
@@ -759,15 +765,15 @@
         <v>4</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E11" s="10">
         <v>1.2</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>2</v>
@@ -776,7 +782,7 @@
         <v>4</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E12" s="10">
         <v>1.2</v>
@@ -784,7 +790,7 @@
     </row>
     <row r="13" spans="1:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>2</v>
@@ -793,7 +799,7 @@
         <v>3</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="E13" s="10">
         <v>4</v>
@@ -801,7 +807,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>2</v>
@@ -810,7 +816,7 @@
         <v>3</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="E14" s="3">
         <v>10001</v>

</xml_diff>